<commit_message>
fixing geo dataissue and adding geoID to templates
</commit_message>
<xml_diff>
--- a/src/test/resources/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
+++ b/src/test/resources/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>List of farmers</t>
   </si>
@@ -125,6 +125,12 @@
   </si>
   <si>
     <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)))</t>
+  </si>
+  <si>
+    <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)), POINT(lat lon), GeoJSON, geoshape de ODK/Kobo "lat lon alt prec;...", o P1(...)P2(...) para varias parcelas)</t>
+  </si>
+  <si>
+    <t>GeoID (FAO) - identificador del límite de la parcela en el registro GeoID de la FAO</t>
   </si>
 </sst>
 </file>
@@ -1544,7 +1550,7 @@
   <dimension ref="A1:AM260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="35" max="40" customWidth="true" style="1" width="8.6640625"/>
+    <col min="36" max="40" customWidth="true" style="1" width="8.6640625"/>
     <col min="1" max="1" customWidth="true" style="1" width="25.33203125"/>
     <col min="2" max="2" customWidth="true" style="1" width="17.0"/>
     <col min="3" max="3" customWidth="true" style="1" width="26.1640625"/>
@@ -1568,6 +1574,7 @@
     <col min="32" max="32" customWidth="true" style="1" width="25.5"/>
     <col min="33" max="33" customWidth="true" style="1" width="22.6640625"/>
     <col min="34" max="34" customWidth="true" style="1" width="29.5703125"/>
+    <col min="35" max="35" customWidth="true" style="1" width="29.5703125"/>
     <col min="41" max="16384" style="1" width="8.6640625"/>
   </cols>
   <sheetData>
@@ -1838,9 +1845,11 @@
         <v>29</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
-      <c r="AI5" s="3"/>
+      <c r="AI5" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>

</xml_diff>